<commit_message>
Sjekkpakker: lenker til K1216–K1223
</commit_message>
<xml_diff>
--- a/dugnad/sjekkpakker/DEM-06.xlsx
+++ b/dugnad/sjekkpakker/DEM-06.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="165">
   <si>
     <t>Sjekkpakke DEM-06: Språk og kultur</t>
   </si>
@@ -518,11 +518,14 @@
     <t>Kultur- og likestillingsdepartementet (2026) – Prop. 41 LS (2025–2026) Endringer i åndsverkloven mv. (gjennomføring av nett- og videresendingsdirektivet og digitalmarkedsdirektivet) · regjeringen.no</t>
   </si>
   <si>
+    <t>https://www.regjeringen.no/no/dokumenter/prop.-41-ls-20252026/id3154279/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Regjeringen ser problemet: språkmodellene som brukes i dag, har «ofte begrenset språklig kvalitet og kulturelle skjevheter», er utviklet av store selskaper i USA og Kina, og det er «usikkert i hvilken grad opphavsrettslige hensyn er ivaretatt ved trening av modellene» [K1219].
 Nasjonalbibliotekets samlinger: pliktavlevert materiale kan brukes til tekst- og datautvinning i forskning, men ikke til kommersielle formål [K1219].</t>
   </si>
   <si>
-    <t>ikke verifisert · Lagt til 2026-10-27 (REG-02). Godkjent i statsråd 27.03.2026. Kap. 4 om tekst- og datautvinning. Sjekk om vedtatt. URL mangler.</t>
+    <t>ikke verifisert · Lagt til 2026-10-27 (REG-02). Godkjent i statsråd 27.03.2026. Kap. 4 om tekst- og datautvinning. Sjekk om vedtatt.</t>
   </si>
 </sst>
 </file>
@@ -1834,14 +1837,14 @@
       <c r="D18" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="E18" s="9" t="s">
-        <v>3</v>
+      <c r="E18" s="10" t="s">
+        <v>162</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
@@ -1901,6 +1904,7 @@
     <hyperlink ref="E14" r:id="rId6"/>
     <hyperlink ref="E15" r:id="rId7"/>
     <hyperlink ref="E16" r:id="rId8"/>
+    <hyperlink ref="E18" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>